<commit_message>
Add Lazada template dropdowns and tab matching
</commit_message>
<xml_diff>
--- a/adapters/lazada-plus-v1/templates/lazada-voucher-template.xlsx
+++ b/adapters/lazada-plus-v1/templates/lazada-voucher-template.xlsx
@@ -8,11 +8,26 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vouchers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FlexiTiers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_枚举值" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FlexiTiers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="Enum_SiteCodes">'_枚举值'!$A$2:$A$7</definedName>
+    <definedName name="Enum_ToolLabels">'_枚举值'!$B$2:$B$5</definedName>
+    <definedName name="Enum_UseTimeTypes">'_枚举值'!$C$2:$C$3</definedName>
+    <definedName name="Enum_ApplyScopes">'_枚举值'!$D$2:$D$3</definedName>
+    <definedName name="Enum_DiscountTypes">'_枚举值'!$E$2:$E$3</definedName>
+    <definedName name="Enum_BudgetModes">'_枚举值'!$F$2:$F$3</definedName>
+    <definedName name="Enum_FlexiMainTypes">'_枚举值'!$G$2:$G$5</definedName>
+    <definedName name="Enum_FlexiCriteriaTypes">'_枚举值'!$H$2:$H$3</definedName>
+    <definedName name="Enum_BooleanFlags">'_枚举值'!$I$2:$I$3</definedName>
+    <definedName name="FlexiSubtype_MONEY_DISCOUNT_OFF">'_枚举值'!$J$2:$J$3</definedName>
+    <definedName name="FlexiSubtype_FREE_GIFT_SAMPLE">'_枚举值'!$K$2:$K$7</definedName>
+    <definedName name="FlexiSubtype_COMBO_BUY">'_枚举值'!$L$2:$L$9</definedName>
+    <definedName name="FlexiSubtype_FIXED_PRICE">'_枚举值'!$M$2:$M$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -978,11 +993,354 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="11">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="站点 请输入下拉列表中的有效枚举值。" promptTitle="站点 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_SiteCodes</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="优惠工具 请输入下拉列表中的有效枚举值。" promptTitle="优惠工具 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_ToolLabels</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="领取生效类型 请输入下拉列表中的有效枚举值。" promptTitle="领取生效类型 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_UseTimeTypes</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="适用范围 请输入下拉列表中的有效枚举值。" promptTitle="适用范围 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_ApplyScopes</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="折扣类型 请输入下拉列表中的有效枚举值。" promptTitle="折扣类型 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_DiscountTypes</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="预算模式 请输入下拉列表中的有效枚举值。" promptTitle="预算模式 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_BudgetModes</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="Flexi主玩法 请输入下拉列表中的有效枚举值。" promptTitle="Flexi主玩法 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_FlexiMainTypes</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="Flexi子玩法 请输入下拉列表中的有效枚举值。" promptTitle="Flexi子玩法 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=INDIRECT("FlexiSubtype_"&amp;$U2)</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="Flexi条件类型 请输入下拉列表中的有效枚举值。" promptTitle="Flexi条件类型 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_FlexiCriteriaTypes</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="Flexi是否叠加折扣 请输入下拉列表中的有效枚举值。" promptTitle="Flexi是否叠加折扣 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_BooleanFlags</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效选项" error="Flexi赠品是否免邮 请输入下拉列表中的有效枚举值。" promptTitle="Flexi赠品是否免邮 可选值" prompt="请优先从下拉框中选择枚举值。" type="list">
+      <formula1>=Enum_BooleanFlags</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Enum_SiteCodes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Enum_ToolLabels</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Enum_UseTimeTypes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Enum_ApplyScopes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Enum_DiscountTypes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Enum_BudgetModes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Enum_FlexiMainTypes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Enum_FlexiCriteriaTypes</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Enum_BooleanFlags</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>FlexiSubtype_MONEY_DISCOUNT_OFF</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FlexiSubtype_FREE_GIFT_SAMPLE</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>FlexiSubtype_COMBO_BUY</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>FlexiSubtype_FIXED_PRICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Regular Voucher</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FIXED_TIME</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ENTIRE_SHOP</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MONEY_OFF</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LIMITED</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>MONEY_DISCOUNT_OFF</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ITEM_QUANTITY</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>MoneyValueOff</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>FreeGiftsOnly</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>MoneyValueOff</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flexi Combo</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USE_AFTER_COLLECTION</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SPECIFIC_PRODUCTS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PERCENT_OFF</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>UNLIMITED</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FREE_GIFT_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ORDER_VALUE</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PercentageDiscountOff</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FreeSamplesOnly</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>PercentageDiscountOff</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Store New Buyer Voucher</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>COMBO_BUY</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PercentOffAndFreeGift</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>FreeGiftsOnly</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Store Follower Voucher</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FIXED_PRICE</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>MoneyOffAndFreeGift</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>FreeSamplesOnly</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>PercentOffAndFreeSample</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>PercentOffAndFreeGift</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>MoneyOffAndFreeSample</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>MoneyOffAndFreeGift</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PercentOffAndFreeSample</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>MoneyOffAndFreeSample</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1108,13 +1466,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1147,12 +1505,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>站点</t>
+          <t>枚举型字段</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>页面右侧国家栏可切换 Indonesia / Malaysia / Philippine / Singapore / Thailand / Vietnam；当前 live 已回归 MY / SG。</t>
+          <t>模板里的站点、优惠工具、领取生效类型、适用范围、折扣类型、预算模式、Flexi 主玩法 / 子玩法 / 条件类型等字段已预置下拉框。</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1522,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>优惠工具</t>
+          <t>站点</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>支持填写 Regular Voucher、Flexi Combo、Store New Buyer Voucher、Store Follower Voucher。</t>
+          <t>页面右侧国家栏可切换 Indonesia / Malaysia / Philippine / Singapore / Thailand / Vietnam；当前 live 已回归 MY / SG。</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1539,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>启用</t>
+          <t>优惠工具</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>已移除。导入模板里的每一行默认都会参与执行。</t>
+          <t>支持填写 Regular Voucher、Flexi Combo、Store New Buyer Voucher、Store Follower Voucher。</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1556,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>领取生效类型</t>
+          <t>启用</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>仅 Voucher 类工具使用；FIXED_TIME 对应固定时间生效，USE_AFTER_COLLECTION 对应领取后生效。</t>
+          <t>已移除。导入模板里的每一行默认都会参与执行。</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1573,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>适用范围</t>
+          <t>领取生效类型</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Specific Products 已完成字段探查，但 live phase 仍需补商品选择。</t>
+          <t>仅 Voucher 类工具使用；FIXED_TIME 对应固定时间生效，USE_AFTER_COLLECTION 对应领取后生效。</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1590,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>预算模式/预算金额</t>
+          <t>适用范围</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>仅 Regular Voucher + MONEY_OFF 使用；Regular 的百分比折扣页面改为总发行量。</t>
+          <t>Specific Products 已完成字段探查，但 live phase 仍需补商品选择。</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1607,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>总发行量</t>
+          <t>预算模式/预算金额</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Store New Buyer / Store Follower 必填；Regular Voucher 的百分比折扣场景也需要填写。</t>
+          <t>仅 Regular Voucher + MONEY_OFF 使用；Regular 的百分比折扣页面改为总发行量。</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1624,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Flexi主玩法</t>
+          <t>总发行量</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Flexi Combo 页面有四张主卡：Money/Discount Off、Free gift/sample、Combo Buy、Fixed Price。</t>
+          <t>Store New Buyer / Store Follower 必填；Regular Voucher 的百分比折扣场景也需要填写。</t>
         </is>
       </c>
     </row>
@@ -1283,29 +1641,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Flexi子玩法</t>
+          <t>Flexi主玩法</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>不同主玩法下可选值不同，详情见 lazada-voucher-field-guide.csv。</t>
+          <t>Flexi Combo 页面有四张主卡：Money/Discount Off、Free gift/sample、Combo Buy、Fixed Price。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FlexiTiers</t>
+          <t>Vouchers</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>唯一键</t>
+          <t>Flexi子玩法</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>必须和 Vouchers sheet 的“唯一键”一致。</t>
+          <t>不同主玩法下可选值不同，详情见 lazada-voucher-field-guide.csv。</t>
         </is>
       </c>
     </row>
@@ -1317,12 +1675,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>门槛值</t>
+          <t>唯一键</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Item Quantity 模式填件数；Order Value 模式填订单金额。</t>
+          <t>必须和 Vouchers sheet 的“唯一键”一致。</t>
         </is>
       </c>
     </row>
@@ -1334,10 +1692,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>门槛值</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Item Quantity 模式填件数；Order Value 模式填订单金额。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FlexiTiers</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>赠品SKU列表</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>当前只做字段固化；live 商品选择弹层后续接入。</t>
         </is>
@@ -1348,7 +1723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix Lazada voucher VN live flow and document ID redirect
</commit_message>
<xml_diff>
--- a/adapters/lazada-plus-v1/templates/lazada-voucher-template.xlsx
+++ b/adapters/lazada-plus-v1/templates/lazada-voucher-template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vouchers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_枚举值" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FlexiTiers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vouchers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_枚举值" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="FlexiTiers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="填写说明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="Enum_SiteCodes">'_枚举值'!$A$2:$A$7</definedName>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>页面右侧国家栏可切换 Indonesia / Malaysia / Philippine / Singapore / Thailand / Vietnam；当前 live 已回归 MY / SG。</t>
+          <t>页面右侧国家栏可切换 Indonesia / Malaysia / Philippine / Singapore / Thailand / Vietnam；当前版本支持六站点切换，建议先按小批量首跑。</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>页面右侧国家栏实测可见 6 个站点；当前 live 已回归 MY / SG。</t>
+          <t>页面右侧国家栏实测可见 6 个站点；当前版本支持六站点切换，建议先按小批量首跑。</t>
         </is>
       </c>
     </row>

</xml_diff>